<commit_message>
Update to latest help and data files
</commit_message>
<xml_diff>
--- a/StatsDirectUI/Assets/Data/test.xlsx
+++ b/StatsDirectUI/Assets/Data/test.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fileVersion appName="SpreadsheetGear 7.0.5.106"/>
+  <fileVersion appName="SpreadsheetGear 7.0.6.138"/>
   <workbookPr defaultThemeVersion="153222"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="17340" windowHeight="11070" tabRatio="757"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1162" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1166" uniqueCount="526">
   <si>
     <t>2nd</t>
   </si>
@@ -1596,6 +1596,12 @@
   </si>
   <si>
     <t>Hgb</t>
+  </si>
+  <si>
+    <t>Serum Creatinine</t>
+  </si>
+  <si>
+    <t>Plasma Creatinine</t>
   </si>
 </sst>
 </file>
@@ -1603,7 +1609,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1618,6 +1624,13 @@
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1637,14 +1650,24 @@
       <name val="Arial"/>
     </font>
     <font>
-      <i/>
       <sz val="10"/>
-      <color rgb="FF7F7F7F"/>
+      <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF7F7F7F"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1656,45 +1679,7 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF006100"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF9C6500"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1706,6 +1691,34 @@
     <font>
       <b/>
       <sz val="10"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF006100"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -1729,7 +1742,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <protection locked="0"/>
@@ -1742,10 +1755,11 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5065,7 +5079,7 @@
       <c s="1">
         <v>2</v>
       </c>
-      <c s="8">
+      <c s="10">
         <v>35490</v>
       </c>
     </row>
@@ -5094,7 +5108,7 @@
       <c s="1">
         <v>1</v>
       </c>
-      <c s="8">
+      <c s="10">
         <v>35552</v>
       </c>
     </row>
@@ -5123,7 +5137,7 @@
       <c s="1">
         <v>1</v>
       </c>
-      <c s="8">
+      <c s="10">
         <v>35411</v>
       </c>
     </row>
@@ -5152,7 +5166,7 @@
       <c s="1">
         <v>0</v>
       </c>
-      <c s="8">
+      <c s="10">
         <v>35370</v>
       </c>
     </row>
@@ -5181,7 +5195,7 @@
       <c s="1">
         <v>2</v>
       </c>
-      <c s="8">
+      <c s="10">
         <v>35433</v>
       </c>
     </row>
@@ -5208,7 +5222,7 @@
       <c s="1">
         <v>1</v>
       </c>
-      <c s="8">
+      <c s="10">
         <v>35555</v>
       </c>
     </row>
@@ -5235,7 +5249,7 @@
       <c s="1">
         <v>0</v>
       </c>
-      <c s="8">
+      <c s="10">
         <v>35649</v>
       </c>
     </row>
@@ -5262,7 +5276,7 @@
       <c s="1">
         <v>2</v>
       </c>
-      <c s="8">
+      <c s="10">
         <v>35346</v>
       </c>
     </row>
@@ -20625,7 +20639,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:CF283"/>
+  <dimension ref="A1:CH283"/>
   <sheetFormatPr defaultColWidth="10.42578125" defaultRowHeight="14.95"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -20691,7 +20705,9 @@
     <col min="74" max="74" width="9" style="2" bestFit="1" customWidth="1"/>
     <col min="75" max="83" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="84" max="84" width="15" style="2" bestFit="1" customWidth="1"/>
-    <col min="85" max="16384" width="10.42578125" style="2"/>
+    <col min="85" max="85" width="15.46875" style="2" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="14.94921875" style="2" bestFit="1" customWidth="1"/>
+    <col min="87" max="16384" width="10.42578125" style="2"/>
   </cols>
   <sheetData>
     <row>
@@ -20947,6 +20963,12 @@
       <c s="2" t="s">
         <v>454</v>
       </c>
+      <c s="8" t="s">
+        <v>525</v>
+      </c>
+      <c s="8" t="s">
+        <v>524</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -21201,6 +21223,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>0.81999999999999995</v>
+      </c>
+      <c s="8">
+        <v>0.79000000000000004</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -21455,6 +21483,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>1.8300000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.6200000000000001</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -21708,6 +21742,12 @@
       </c>
       <c s="2">
         <v>0</v>
+      </c>
+      <c s="8">
+        <v>1.3899999999999999</v>
+      </c>
+      <c s="8">
+        <v>1.3600000000000001</v>
       </c>
     </row>
     <row>
@@ -21957,6 +21997,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>0.81000000000000005</v>
+      </c>
+      <c s="8">
+        <v>1.3</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -22205,6 +22251,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>1.72</v>
+      </c>
+      <c s="8">
+        <v>1.8799999999999999</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -22447,6 +22499,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>3.23</v>
+      </c>
+      <c s="8">
+        <v>3.3500000000000001</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -22668,6 +22726,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>1.23</v>
+      </c>
+      <c s="8">
+        <v>1.0600000000000001</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -22889,6 +22953,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>1.3700000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.3400000000000001</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -23092,6 +23162,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>1.72</v>
+      </c>
+      <c s="8">
+        <v>1.5600000000000001</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -23295,6 +23371,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>0.95999999999999996</v>
+      </c>
+      <c s="8">
+        <v>0.93999999999999995</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -23489,6 +23571,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c s="8">
+        <v>0.76000000000000001</v>
+      </c>
+      <c s="8">
+        <v>0.68999999999999995</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -23683,6 +23771,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>1.1499999999999999</v>
+      </c>
+      <c s="8">
+        <v>1.1599999999999999</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -23859,6 +23953,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>0.94999999999999996</v>
+      </c>
+      <c s="8">
+        <v>0.70999999999999996</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -24032,6 +24132,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>1</v>
+      </c>
+      <c s="8">
+        <v>0.82999999999999996</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -24190,6 +24296,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>1.52</v>
+      </c>
+      <c s="8">
+        <v>1.4399999999999999</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -24348,6 +24460,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>1.5600000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.26</v>
+      </c>
     </row>
     <row>
       <c r="M18" s="1">
@@ -24485,6 +24603,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>2.4500000000000002</v>
+      </c>
+      <c s="8">
+        <v>2.3599999999999999</v>
+      </c>
     </row>
     <row>
       <c r="M19" s="1">
@@ -24622,6 +24746,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>1.8500000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.8999999999999999</v>
+      </c>
     </row>
     <row>
       <c r="M20" s="1">
@@ -24759,6 +24889,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>0.89000000000000001</v>
+      </c>
+      <c s="8">
+        <v>0.94999999999999996</v>
+      </c>
     </row>
     <row>
       <c r="M21" s="1">
@@ -24896,6 +25032,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>0.81999999999999995</v>
+      </c>
+      <c s="8">
+        <v>0.77000000000000002</v>
+      </c>
     </row>
     <row>
       <c r="M22" s="1">
@@ -25033,6 +25175,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c s="8">
+        <v>1.01</v>
+      </c>
+      <c s="8">
+        <v>0.81999999999999995</v>
+      </c>
     </row>
     <row>
       <c r="M23" s="1">
@@ -25170,6 +25318,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c s="8">
+        <v>0.95999999999999996</v>
+      </c>
+      <c s="8">
+        <v>0.88</v>
+      </c>
     </row>
     <row>
       <c r="M24" s="1">
@@ -25262,6 +25416,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG24" s="8">
+        <v>3.3799999999999999</v>
+      </c>
+      <c s="8">
+        <v>3.4199999999999999</v>
+      </c>
     </row>
     <row>
       <c r="M25" s="1">
@@ -25354,6 +25514,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG25" s="8">
+        <v>1.3100000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.1499999999999999</v>
+      </c>
     </row>
     <row>
       <c r="M26" s="1">
@@ -25446,6 +25612,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG26" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c s="8">
+        <v>0.95999999999999996</v>
+      </c>
     </row>
     <row>
       <c r="M27" s="1">
@@ -25529,6 +25701,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG27" s="8">
+        <v>1.26</v>
+      </c>
+      <c s="8">
+        <v>1.1200000000000001</v>
+      </c>
     </row>
     <row>
       <c r="M28" s="1">
@@ -25609,6 +25787,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG28" s="8">
+        <v>1.1499999999999999</v>
+      </c>
+      <c s="8">
+        <v>1.02</v>
+      </c>
     </row>
     <row>
       <c r="M29" s="1">
@@ -25689,6 +25873,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG29" s="8">
+        <v>1.2</v>
+      </c>
+      <c s="8">
+        <v>1.29</v>
+      </c>
     </row>
     <row>
       <c r="M30" s="1">
@@ -25763,6 +25953,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG30" s="8">
+        <v>1.01</v>
+      </c>
+      <c s="8">
+        <v>0.87</v>
+      </c>
     </row>
     <row>
       <c r="M31" s="1">
@@ -25837,6 +26033,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG31" s="8">
+        <v>1.3300000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.1299999999999999</v>
+      </c>
     </row>
     <row>
       <c r="M32" s="1">
@@ -25911,6 +26113,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG32" s="8">
+        <v>0.87</v>
+      </c>
+      <c s="8">
+        <v>0.81999999999999995</v>
+      </c>
     </row>
     <row>
       <c r="M33" s="1">
@@ -25985,6 +26193,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG33" s="8">
+        <v>1.6599999999999999</v>
+      </c>
+      <c s="8">
+        <v>1.3300000000000001</v>
+      </c>
     </row>
     <row>
       <c r="O34" s="1">
@@ -26053,6 +26267,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG34" s="8">
+        <v>1.4099999999999999</v>
+      </c>
+      <c s="8">
+        <v>1.1399999999999999</v>
+      </c>
     </row>
     <row>
       <c r="O35" s="1">
@@ -26121,6 +26341,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG35" s="8">
+        <v>1.0800000000000001</v>
+      </c>
+      <c s="8">
+        <v>0.93000000000000005</v>
+      </c>
     </row>
     <row>
       <c r="O36" s="1">
@@ -26189,6 +26415,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG36" s="8">
+        <v>1.1699999999999999</v>
+      </c>
+      <c s="8">
+        <v>1.0900000000000001</v>
+      </c>
     </row>
     <row>
       <c r="O37" s="1">
@@ -26257,6 +26489,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG37" s="8">
+        <v>1.77</v>
+      </c>
+      <c s="8">
+        <v>1.8899999999999999</v>
+      </c>
     </row>
     <row>
       <c r="O38" s="1">
@@ -26325,6 +26563,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG38" s="8">
+        <v>1.3300000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.5700000000000001</v>
+      </c>
     </row>
     <row>
       <c r="O39" s="1">
@@ -26393,6 +26637,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG39" s="8">
+        <v>1.23</v>
+      </c>
+      <c s="8">
+        <v>1.29</v>
+      </c>
     </row>
     <row>
       <c r="O40" s="1">
@@ -26461,6 +26711,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG40" s="8">
+        <v>1.21</v>
+      </c>
+      <c s="8">
+        <v>1.1299999999999999</v>
+      </c>
     </row>
     <row>
       <c r="O41" s="1">
@@ -26529,6 +26785,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG41" s="8">
+        <v>1.2</v>
+      </c>
+      <c s="8">
+        <v>1.1100000000000001</v>
+      </c>
     </row>
     <row>
       <c r="O42" s="1">
@@ -26597,6 +26859,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG42" s="8">
+        <v>1.49</v>
+      </c>
+      <c s="8">
+        <v>1.6100000000000001</v>
+      </c>
     </row>
     <row>
       <c r="O43" s="1">
@@ -26665,6 +26933,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG43" s="8">
+        <v>0.89000000000000001</v>
+      </c>
+      <c s="8">
+        <v>0.79000000000000004</v>
+      </c>
     </row>
     <row>
       <c r="O44" s="1">
@@ -26733,6 +27007,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG44" s="8">
+        <v>1.0900000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.1899999999999999</v>
+      </c>
     </row>
     <row>
       <c r="O45" s="1">
@@ -26801,6 +27081,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG45" s="8">
+        <v>1.03</v>
+      </c>
+      <c s="8">
+        <v>0.95999999999999996</v>
+      </c>
     </row>
     <row>
       <c r="O46" s="1">
@@ -26863,6 +27149,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG46" s="8">
+        <v>1.0700000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.25</v>
+      </c>
     </row>
     <row>
       <c r="O47" s="1">
@@ -26925,6 +27217,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG47" s="8">
+        <v>0.89000000000000001</v>
+      </c>
+      <c s="8">
+        <v>0.87</v>
+      </c>
     </row>
     <row>
       <c r="O48" s="1">
@@ -26987,6 +27285,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG48" s="8">
+        <v>1.3899999999999999</v>
+      </c>
+      <c s="8">
+        <v>1.3600000000000001</v>
+      </c>
     </row>
     <row>
       <c r="O49" s="1">
@@ -27049,6 +27353,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG49" s="8">
+        <v>0.95999999999999996</v>
+      </c>
+      <c s="8">
+        <v>0.85999999999999999</v>
+      </c>
     </row>
     <row>
       <c r="O50" s="1">
@@ -27111,6 +27421,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG50" s="8">
+        <v>1.0600000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.03</v>
+      </c>
     </row>
     <row>
       <c r="O51" s="1">
@@ -27173,6 +27489,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG51" s="8">
+        <v>1.1699999999999999</v>
+      </c>
+      <c s="8">
+        <v>0.85999999999999999</v>
+      </c>
     </row>
     <row>
       <c r="O52" s="1">
@@ -27235,6 +27557,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG52" s="8">
+        <v>0.90000000000000002</v>
+      </c>
+      <c s="8">
+        <v>0.80000000000000004</v>
+      </c>
     </row>
     <row>
       <c r="O53" s="1">
@@ -27297,6 +27625,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG53" s="8">
+        <v>1.3899999999999999</v>
+      </c>
+      <c s="8">
+        <v>1.22</v>
+      </c>
     </row>
     <row>
       <c r="O54" s="1">
@@ -27359,6 +27693,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG54" s="8">
+        <v>0.91000000000000003</v>
+      </c>
+      <c s="8">
+        <v>0.85999999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP55" s="1">
@@ -27412,6 +27752,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG55" s="8">
+        <v>2.2799999999999998</v>
+      </c>
+      <c s="8">
+        <v>2.25</v>
+      </c>
     </row>
     <row>
       <c r="AP56" s="1">
@@ -27465,6 +27811,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG56" s="8">
+        <v>0.90000000000000002</v>
+      </c>
+      <c s="8">
+        <v>0.87</v>
+      </c>
     </row>
     <row>
       <c r="AP57" s="1">
@@ -27518,6 +27870,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG57" s="8">
+        <v>1.3400000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.3</v>
+      </c>
     </row>
     <row>
       <c r="AP58" s="1">
@@ -27571,6 +27929,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG58" s="8">
+        <v>1.3200000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.04</v>
+      </c>
     </row>
     <row>
       <c r="AP59" s="1">
@@ -27624,6 +27988,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG59" s="8">
+        <v>1.02</v>
+      </c>
+      <c s="8">
+        <v>0.92000000000000004</v>
+      </c>
     </row>
     <row>
       <c r="AP60" s="1">
@@ -27677,6 +28047,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG60" s="8">
+        <v>1.04</v>
+      </c>
+      <c s="8">
+        <v>1.01</v>
+      </c>
     </row>
     <row>
       <c r="AP61" s="1">
@@ -27730,6 +28106,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG61" s="8">
+        <v>1.27</v>
+      </c>
+      <c s="8">
+        <v>1.21</v>
+      </c>
     </row>
     <row>
       <c r="AP62" s="1">
@@ -27783,6 +28165,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG62" s="8">
+        <v>1.0800000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.1100000000000001</v>
+      </c>
     </row>
     <row>
       <c r="AP63" s="1">
@@ -27836,6 +28224,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG63" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.21</v>
+      </c>
     </row>
     <row>
       <c r="AP64" s="1">
@@ -27889,6 +28283,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG64" s="8">
+        <v>1.3899999999999999</v>
+      </c>
+      <c s="8">
+        <v>1.54</v>
+      </c>
     </row>
     <row>
       <c r="AP65" s="1">
@@ -27942,6 +28342,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG65" s="8">
+        <v>1.0700000000000001</v>
+      </c>
+      <c s="8">
+        <v>0.98999999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP66" s="1">
@@ -27995,6 +28401,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG66" s="8">
+        <v>0.79000000000000004</v>
+      </c>
+      <c s="8">
+        <v>0.79000000000000004</v>
+      </c>
     </row>
     <row>
       <c r="AP67" s="1">
@@ -28048,6 +28460,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG67" s="8">
+        <v>1.02</v>
+      </c>
+      <c s="8">
+        <v>1.0600000000000001</v>
+      </c>
     </row>
     <row>
       <c r="AP68" s="1">
@@ -28101,6 +28519,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG68" s="8">
+        <v>0.93999999999999995</v>
+      </c>
+      <c s="8">
+        <v>1.02</v>
+      </c>
     </row>
     <row>
       <c r="AP69" s="1">
@@ -28154,6 +28578,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG69" s="8">
+        <v>1.99</v>
+      </c>
+      <c s="8">
+        <v>2.1499999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP70" s="1">
@@ -28207,6 +28637,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG70" s="8">
+        <v>0.69999999999999996</v>
+      </c>
+      <c s="8">
+        <v>0.56000000000000005</v>
+      </c>
     </row>
     <row>
       <c r="AP71" s="1">
@@ -28260,6 +28696,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG71" s="8">
+        <v>0.83999999999999997</v>
+      </c>
+      <c s="8">
+        <v>1.01</v>
+      </c>
     </row>
     <row>
       <c r="AP72" s="1">
@@ -28313,6 +28755,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG72" s="8">
+        <v>0.66000000000000003</v>
+      </c>
+      <c s="8">
+        <v>0.58999999999999997</v>
+      </c>
     </row>
     <row>
       <c r="AP73" s="1">
@@ -28366,6 +28814,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG73" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.1699999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP74" s="1">
@@ -28419,6 +28873,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG74" s="8">
+        <v>0.90000000000000002</v>
+      </c>
+      <c s="8">
+        <v>0.81999999999999995</v>
+      </c>
     </row>
     <row>
       <c r="AP75" s="1">
@@ -28472,6 +28932,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG75" s="8">
+        <v>2.0600000000000001</v>
+      </c>
+      <c s="8">
+        <v>2.0899999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP76" s="1">
@@ -28525,6 +28991,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG76" s="8">
+        <v>1.3100000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.4399999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP77" s="1">
@@ -28578,6 +29050,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG77" s="8">
+        <v>1.03</v>
+      </c>
+      <c s="8">
+        <v>1.22</v>
+      </c>
     </row>
     <row>
       <c r="AP78" s="1">
@@ -28631,6 +29109,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG78" s="8">
+        <v>1.6100000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.77</v>
+      </c>
     </row>
     <row>
       <c r="AP79" s="1">
@@ -28684,6 +29168,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG79" s="8">
+        <v>1.52</v>
+      </c>
+      <c s="8">
+        <v>1.6000000000000001</v>
+      </c>
     </row>
     <row>
       <c r="AP80" s="1">
@@ -28737,6 +29227,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG80" s="8">
+        <v>1.1100000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.1299999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP81" s="1">
@@ -28790,6 +29286,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG81" s="8">
+        <v>0.84999999999999998</v>
+      </c>
+      <c s="8">
+        <v>1.0600000000000001</v>
+      </c>
     </row>
     <row>
       <c r="AP82" s="1">
@@ -28843,6 +29345,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG82" s="8">
+        <v>1.2</v>
+      </c>
+      <c s="8">
+        <v>1.3799999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP83" s="1">
@@ -28896,6 +29404,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG83" s="8">
+        <v>1.0900000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.24</v>
+      </c>
     </row>
     <row>
       <c r="AP84" s="1">
@@ -28949,6 +29463,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG84" s="8">
+        <v>1.27</v>
+      </c>
+      <c s="8">
+        <v>1.29</v>
+      </c>
     </row>
     <row>
       <c r="AP85" s="1">
@@ -29002,6 +29522,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG85" s="8">
+        <v>2.0600000000000001</v>
+      </c>
+      <c s="8">
+        <v>2.0800000000000001</v>
+      </c>
     </row>
     <row>
       <c r="AP86" s="1">
@@ -29055,6 +29581,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG86" s="8">
+        <v>1.21</v>
+      </c>
+      <c s="8">
+        <v>1.3100000000000001</v>
+      </c>
     </row>
     <row>
       <c r="AP87" s="1">
@@ -29108,6 +29640,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG87" s="8">
+        <v>0.77000000000000002</v>
+      </c>
+      <c s="8">
+        <v>0.81999999999999995</v>
+      </c>
     </row>
     <row>
       <c r="AP88" s="1">
@@ -29161,6 +29699,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG88" s="8">
+        <v>1.0600000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.28</v>
+      </c>
     </row>
     <row>
       <c r="AP89" s="1">
@@ -29214,6 +29758,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG89" s="8">
+        <v>1.02</v>
+      </c>
+      <c s="8">
+        <v>1.1499999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP90" s="1">
@@ -29267,6 +29817,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG90" s="8">
+        <v>1</v>
+      </c>
+      <c s="8">
+        <v>1.04</v>
+      </c>
     </row>
     <row>
       <c r="AP91" s="1">
@@ -29320,6 +29876,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG91" s="8">
+        <v>1.47</v>
+      </c>
+      <c s="8">
+        <v>1.51</v>
+      </c>
     </row>
     <row>
       <c r="AP92" s="1">
@@ -29373,6 +29935,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG92" s="8">
+        <v>0.96999999999999997</v>
+      </c>
+      <c s="8">
+        <v>1.1299999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP93" s="1">
@@ -29426,6 +29994,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG93" s="8">
+        <v>1.7</v>
+      </c>
+      <c s="8">
+        <v>1.8400000000000001</v>
+      </c>
     </row>
     <row>
       <c r="AP94" s="1">
@@ -29479,6 +30053,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG94" s="8">
+        <v>1.78</v>
+      </c>
+      <c s="8">
+        <v>1.9399999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP95" s="1">
@@ -29532,6 +30112,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG95" s="8">
+        <v>0.93000000000000005</v>
+      </c>
+      <c s="8">
+        <v>1.3200000000000001</v>
+      </c>
     </row>
     <row>
       <c r="AP96" s="1">
@@ -29585,6 +30171,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG96" s="8">
+        <v>0.92000000000000004</v>
+      </c>
+      <c s="8">
+        <v>1.3600000000000001</v>
+      </c>
     </row>
     <row>
       <c r="AP97" s="1">
@@ -29638,6 +30230,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG97" s="8">
+        <v>1.5900000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.8799999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP98" s="1">
@@ -29691,6 +30289,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG98" s="8">
+        <v>0.68000000000000005</v>
+      </c>
+      <c s="8">
+        <v>0.72999999999999998</v>
+      </c>
     </row>
     <row>
       <c r="AP99" s="1">
@@ -29744,6 +30348,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG99" s="8">
+        <v>0.69999999999999996</v>
+      </c>
+      <c s="8">
+        <v>0.78000000000000003</v>
+      </c>
     </row>
     <row>
       <c r="AP100" s="1">
@@ -29797,6 +30407,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG100" s="8">
+        <v>1.0800000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.01</v>
+      </c>
     </row>
     <row>
       <c r="AP101" s="1">
@@ -29850,6 +30466,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG101" s="8">
+        <v>0.82999999999999996</v>
+      </c>
+      <c s="8">
+        <v>0.90000000000000002</v>
+      </c>
     </row>
     <row>
       <c r="AP102" s="1">
@@ -29903,6 +30525,12 @@
       <c s="2">
         <v>0</v>
       </c>
+      <c r="CG102" s="8">
+        <v>1.1699999999999999</v>
+      </c>
+      <c s="8">
+        <v>1.3</v>
+      </c>
     </row>
     <row>
       <c r="AP103" s="1">
@@ -29956,6 +30584,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG103" s="8">
+        <v>0.97999999999999998</v>
+      </c>
+      <c s="8">
+        <v>0.95999999999999996</v>
+      </c>
     </row>
     <row>
       <c r="AP104" s="1">
@@ -30009,6 +30643,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG104" s="8">
+        <v>0.77000000000000002</v>
+      </c>
+      <c s="8">
+        <v>0.60999999999999999</v>
+      </c>
     </row>
     <row>
       <c r="AP105" s="1">
@@ -30062,6 +30702,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG105" s="8">
+        <v>0.91000000000000003</v>
+      </c>
+      <c s="8">
+        <v>1.27</v>
+      </c>
     </row>
     <row>
       <c r="AP106" s="1">
@@ -30115,6 +30761,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG106" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c s="8">
+        <v>1.05</v>
+      </c>
     </row>
     <row>
       <c r="AP107" s="1">
@@ -30168,6 +30820,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG107" s="8">
+        <v>0.80000000000000004</v>
+      </c>
+      <c s="8">
+        <v>1.1200000000000001</v>
+      </c>
     </row>
     <row>
       <c r="AP108" s="1">
@@ -30221,6 +30879,12 @@
       <c s="2">
         <v>1</v>
       </c>
+      <c r="CG108" s="8">
+        <v>0.84999999999999998</v>
+      </c>
+      <c s="8">
+        <v>0.71999999999999997</v>
+      </c>
     </row>
     <row>
       <c r="AP109" s="1">
@@ -30273,6 +30937,12 @@
       </c>
       <c s="2">
         <v>1</v>
+      </c>
+      <c r="CG109" s="8">
+        <v>0.81999999999999995</v>
+      </c>
+      <c s="8">
+        <v>0.87</v>
       </c>
     </row>
     <row>
@@ -32849,7 +33519,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AH61"/>
+  <dimension ref="A1:AJ109"/>
   <sheetFormatPr defaultRowHeight="14.95"/>
   <cols>
     <col min="1" max="1" width="9" style="2" bestFit="1" customWidth="1"/>
@@ -32874,7 +33544,8 @@
     <col min="32" max="32" width="6.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="8.84375" style="2" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="10.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="11.42578125" style="2" customWidth="1"/>
+    <col min="35" max="35" width="14.94921875" style="2" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="15.46875" style="2" bestFit="1" customWidth="1"/>
     <col min="37" max="16384" width="8.84375" style="2"/>
   </cols>
   <sheetData>
@@ -32981,6 +33652,12 @@
       <c s="2" t="s">
         <v>420</v>
       </c>
+      <c s="2" t="s">
+        <v>524</v>
+      </c>
+      <c s="2" t="s">
+        <v>525</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -33085,6 +33762,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>0.81999999999999995</v>
+      </c>
+      <c s="2">
+        <v>0.79000000000000004</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -33189,6 +33872,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>1.8300000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.6200000000000001</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -33293,6 +33982,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>1.3899999999999999</v>
+      </c>
+      <c s="2">
+        <v>1.3600000000000001</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -33397,6 +34092,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>0.81000000000000005</v>
+      </c>
+      <c s="2">
+        <v>1.3</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -33501,6 +34202,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>1.72</v>
+      </c>
+      <c s="2">
+        <v>1.8799999999999999</v>
+      </c>
     </row>
     <row>
       <c r="F7" s="2">
@@ -33590,6 +34297,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>3.23</v>
+      </c>
+      <c s="2">
+        <v>3.3500000000000001</v>
+      </c>
     </row>
     <row>
       <c r="F8" s="2">
@@ -33679,6 +34392,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>1.23</v>
+      </c>
+      <c s="2">
+        <v>1.0600000000000001</v>
+      </c>
     </row>
     <row>
       <c r="F9" s="2">
@@ -33768,6 +34487,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>1.3700000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.3400000000000001</v>
+      </c>
     </row>
     <row>
       <c r="F10" s="2">
@@ -33857,6 +34582,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>1.72</v>
+      </c>
+      <c s="2">
+        <v>1.5600000000000001</v>
+      </c>
     </row>
     <row>
       <c r="F11" s="2">
@@ -33945,6 +34676,12 @@
       </c>
       <c s="2" t="s">
         <v>118</v>
+      </c>
+      <c s="2">
+        <v>0.95999999999999996</v>
+      </c>
+      <c s="2">
+        <v>0.93999999999999995</v>
       </c>
     </row>
     <row>
@@ -34020,6 +34757,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>0.76000000000000001</v>
+      </c>
+      <c s="2">
+        <v>0.68999999999999995</v>
+      </c>
     </row>
     <row>
       <c r="F13" s="2">
@@ -34094,6 +34837,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1.1499999999999999</v>
+      </c>
+      <c s="2">
+        <v>1.1599999999999999</v>
+      </c>
     </row>
     <row>
       <c r="F14" s="2">
@@ -34168,6 +34917,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>0.94999999999999996</v>
+      </c>
+      <c s="2">
+        <v>0.70999999999999996</v>
+      </c>
     </row>
     <row>
       <c r="F15" s="2">
@@ -34242,6 +34997,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1</v>
+      </c>
+      <c s="2">
+        <v>0.82999999999999996</v>
+      </c>
     </row>
     <row>
       <c r="F16" s="2">
@@ -34316,6 +35077,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1.52</v>
+      </c>
+      <c s="2">
+        <v>1.4399999999999999</v>
+      </c>
     </row>
     <row>
       <c r="F17" s="2">
@@ -34390,6 +35157,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>1.5600000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.26</v>
+      </c>
     </row>
     <row>
       <c r="F18" s="2">
@@ -34464,6 +35237,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>2.4500000000000002</v>
+      </c>
+      <c s="2">
+        <v>2.3599999999999999</v>
+      </c>
     </row>
     <row>
       <c r="F19" s="2">
@@ -34538,6 +35317,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>1.8500000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.8999999999999999</v>
+      </c>
     </row>
     <row>
       <c r="F20" s="2">
@@ -34612,6 +35397,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>0.89000000000000001</v>
+      </c>
+      <c s="2">
+        <v>0.94999999999999996</v>
+      </c>
     </row>
     <row>
       <c r="F21" s="2">
@@ -34686,6 +35477,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>0.81999999999999995</v>
+      </c>
+      <c s="2">
+        <v>0.77000000000000002</v>
+      </c>
     </row>
     <row>
       <c r="F22" s="2">
@@ -34748,6 +35545,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>1.01</v>
+      </c>
+      <c s="2">
+        <v>0.81999999999999995</v>
+      </c>
     </row>
     <row>
       <c r="F23" s="2">
@@ -34810,6 +35613,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>0.95999999999999996</v>
+      </c>
+      <c s="2">
+        <v>0.88</v>
+      </c>
     </row>
     <row>
       <c r="F24" s="2">
@@ -34872,6 +35681,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>3.3799999999999999</v>
+      </c>
+      <c s="2">
+        <v>3.4199999999999999</v>
+      </c>
     </row>
     <row>
       <c r="F25" s="2">
@@ -34913,6 +35728,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>1.3100000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.1499999999999999</v>
+      </c>
     </row>
     <row>
       <c r="F26" s="2">
@@ -34954,6 +35775,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c s="2">
+        <v>0.95999999999999996</v>
+      </c>
     </row>
     <row>
       <c r="T27" s="3">
@@ -34980,6 +35807,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1.26</v>
+      </c>
+      <c s="2">
+        <v>1.1200000000000001</v>
+      </c>
     </row>
     <row>
       <c r="T28" s="3">
@@ -35006,6 +35839,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1.1499999999999999</v>
+      </c>
+      <c s="2">
+        <v>1.02</v>
+      </c>
     </row>
     <row>
       <c r="T29" s="3">
@@ -35032,6 +35871,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1.2</v>
+      </c>
+      <c s="2">
+        <v>1.29</v>
+      </c>
     </row>
     <row>
       <c r="T30" s="3">
@@ -35058,6 +35903,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1.01</v>
+      </c>
+      <c s="2">
+        <v>0.87</v>
+      </c>
     </row>
     <row>
       <c r="T31" s="3">
@@ -35084,6 +35935,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1.3300000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.1299999999999999</v>
+      </c>
     </row>
     <row>
       <c r="T32" s="3">
@@ -35110,6 +35967,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>0.87</v>
+      </c>
+      <c s="2">
+        <v>0.81999999999999995</v>
+      </c>
     </row>
     <row>
       <c r="T33" s="3">
@@ -35136,6 +35999,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>1.6599999999999999</v>
+      </c>
+      <c s="2">
+        <v>1.3300000000000001</v>
+      </c>
     </row>
     <row>
       <c r="T34" s="3">
@@ -35162,6 +36031,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>1.4099999999999999</v>
+      </c>
+      <c s="2">
+        <v>1.1399999999999999</v>
+      </c>
     </row>
     <row>
       <c r="T35" s="3">
@@ -35188,6 +36063,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>1.0800000000000001</v>
+      </c>
+      <c s="2">
+        <v>0.93000000000000005</v>
+      </c>
     </row>
     <row>
       <c r="T36" s="3">
@@ -35214,6 +36095,12 @@
       <c s="2" t="s">
         <v>149</v>
       </c>
+      <c s="2">
+        <v>1.1699999999999999</v>
+      </c>
+      <c s="2">
+        <v>1.0900000000000001</v>
+      </c>
     </row>
     <row>
       <c r="T37" s="3">
@@ -35240,6 +36127,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>1.77</v>
+      </c>
+      <c s="2">
+        <v>1.8899999999999999</v>
+      </c>
     </row>
     <row>
       <c r="T38" s="3">
@@ -35266,6 +36159,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>1.3300000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.5700000000000001</v>
+      </c>
     </row>
     <row>
       <c r="T39" s="3">
@@ -35292,6 +36191,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>1.23</v>
+      </c>
+      <c s="2">
+        <v>1.29</v>
+      </c>
     </row>
     <row>
       <c r="T40" s="3">
@@ -35318,6 +36223,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>1.21</v>
+      </c>
+      <c s="2">
+        <v>1.1299999999999999</v>
+      </c>
     </row>
     <row>
       <c r="T41" s="3">
@@ -35344,6 +36255,12 @@
       <c s="2" t="s">
         <v>118</v>
       </c>
+      <c s="2">
+        <v>1.2</v>
+      </c>
+      <c s="2">
+        <v>1.1100000000000001</v>
+      </c>
     </row>
     <row>
       <c r="T42" s="3">
@@ -35370,6 +36287,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1.49</v>
+      </c>
+      <c s="2">
+        <v>1.6100000000000001</v>
+      </c>
     </row>
     <row>
       <c r="T43" s="3">
@@ -35396,6 +36319,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>0.89000000000000001</v>
+      </c>
+      <c s="2">
+        <v>0.79000000000000004</v>
+      </c>
     </row>
     <row>
       <c r="T44" s="3">
@@ -35422,6 +36351,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1.0900000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.1899999999999999</v>
+      </c>
     </row>
     <row>
       <c r="T45" s="3">
@@ -35448,6 +36383,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1.03</v>
+      </c>
+      <c s="2">
+        <v>0.95999999999999996</v>
+      </c>
     </row>
     <row>
       <c r="T46" s="3">
@@ -35474,6 +36415,12 @@
       <c s="2" t="s">
         <v>345</v>
       </c>
+      <c s="2">
+        <v>1.0700000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.25</v>
+      </c>
     </row>
     <row>
       <c r="T47" s="3">
@@ -35488,6 +36435,12 @@
       <c s="3">
         <v>4</v>
       </c>
+      <c r="AI47" s="2">
+        <v>0.89000000000000001</v>
+      </c>
+      <c s="2">
+        <v>0.87</v>
+      </c>
     </row>
     <row>
       <c r="T48" s="3">
@@ -35502,6 +36455,12 @@
       <c s="3">
         <v>5</v>
       </c>
+      <c r="AI48" s="2">
+        <v>1.3899999999999999</v>
+      </c>
+      <c s="2">
+        <v>1.3600000000000001</v>
+      </c>
     </row>
     <row>
       <c r="T49" s="3">
@@ -35516,6 +36475,12 @@
       <c s="3">
         <v>4</v>
       </c>
+      <c r="AI49" s="2">
+        <v>0.95999999999999996</v>
+      </c>
+      <c s="2">
+        <v>0.85999999999999999</v>
+      </c>
     </row>
     <row>
       <c r="T50" s="3">
@@ -35530,6 +36495,12 @@
       <c s="3">
         <v>4</v>
       </c>
+      <c r="AI50" s="2">
+        <v>1.0600000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.03</v>
+      </c>
     </row>
     <row>
       <c r="T51" s="3">
@@ -35544,6 +36515,12 @@
       <c s="3">
         <v>4</v>
       </c>
+      <c r="AI51" s="2">
+        <v>1.1699999999999999</v>
+      </c>
+      <c s="2">
+        <v>0.85999999999999999</v>
+      </c>
     </row>
     <row>
       <c r="T52" s="3">
@@ -35558,6 +36535,12 @@
       <c s="3">
         <v>4</v>
       </c>
+      <c r="AI52" s="2">
+        <v>0.90000000000000002</v>
+      </c>
+      <c s="2">
+        <v>0.80000000000000004</v>
+      </c>
     </row>
     <row>
       <c r="T53" s="3">
@@ -35572,6 +36555,12 @@
       <c s="3">
         <v>4</v>
       </c>
+      <c r="AI53" s="2">
+        <v>1.3899999999999999</v>
+      </c>
+      <c s="2">
+        <v>1.22</v>
+      </c>
     </row>
     <row>
       <c r="T54" s="3">
@@ -35585,6 +36574,12 @@
       </c>
       <c s="3">
         <v>5</v>
+      </c>
+      <c r="AI54" s="2">
+        <v>0.91000000000000003</v>
+      </c>
+      <c s="2">
+        <v>0.85999999999999999</v>
       </c>
     </row>
     <row>
@@ -35600,6 +36595,12 @@
       <c s="3">
         <v>5</v>
       </c>
+      <c r="AI55" s="2">
+        <v>2.2799999999999998</v>
+      </c>
+      <c s="2">
+        <v>2.25</v>
+      </c>
     </row>
     <row>
       <c r="T56" s="3">
@@ -35614,6 +36615,12 @@
       <c s="3">
         <v>5</v>
       </c>
+      <c r="AI56" s="2">
+        <v>0.90000000000000002</v>
+      </c>
+      <c s="2">
+        <v>0.87</v>
+      </c>
     </row>
     <row>
       <c r="T57" s="3">
@@ -35628,6 +36635,12 @@
       <c s="3">
         <v>4</v>
       </c>
+      <c r="AI57" s="2">
+        <v>1.3400000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.3</v>
+      </c>
     </row>
     <row>
       <c r="T58" s="3">
@@ -35642,6 +36655,12 @@
       <c s="3">
         <v>5</v>
       </c>
+      <c r="AI58" s="2">
+        <v>1.3200000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.04</v>
+      </c>
     </row>
     <row>
       <c r="T59" s="3">
@@ -35656,6 +36675,12 @@
       <c s="3">
         <v>4</v>
       </c>
+      <c r="AI59" s="2">
+        <v>1.02</v>
+      </c>
+      <c s="2">
+        <v>0.92000000000000004</v>
+      </c>
     </row>
     <row>
       <c r="T60" s="3">
@@ -35670,6 +36695,12 @@
       <c s="3">
         <v>4</v>
       </c>
+      <c r="AI60" s="2">
+        <v>1.04</v>
+      </c>
+      <c s="2">
+        <v>1.01</v>
+      </c>
     </row>
     <row>
       <c r="T61" s="3">
@@ -35683,6 +36714,396 @@
       </c>
       <c s="3">
         <v>5</v>
+      </c>
+      <c r="AI61" s="2">
+        <v>1.27</v>
+      </c>
+      <c s="2">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI62" s="2">
+        <v>1.0800000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.1100000000000001</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI63" s="2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI64" s="2">
+        <v>1.3899999999999999</v>
+      </c>
+      <c s="2">
+        <v>1.54</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI65" s="2">
+        <v>1.0700000000000001</v>
+      </c>
+      <c s="2">
+        <v>0.98999999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI66" s="2">
+        <v>0.79000000000000004</v>
+      </c>
+      <c s="2">
+        <v>0.79000000000000004</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI67" s="2">
+        <v>1.02</v>
+      </c>
+      <c s="2">
+        <v>1.0600000000000001</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI68" s="2">
+        <v>0.93999999999999995</v>
+      </c>
+      <c s="2">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI69" s="2">
+        <v>1.99</v>
+      </c>
+      <c s="2">
+        <v>2.1499999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI70" s="2">
+        <v>0.69999999999999996</v>
+      </c>
+      <c s="2">
+        <v>0.56000000000000005</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI71" s="2">
+        <v>0.83999999999999997</v>
+      </c>
+      <c s="2">
+        <v>1.01</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI72" s="2">
+        <v>0.66000000000000003</v>
+      </c>
+      <c s="2">
+        <v>0.58999999999999997</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI73" s="2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.1699999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI74" s="2">
+        <v>0.90000000000000002</v>
+      </c>
+      <c s="2">
+        <v>0.81999999999999995</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI75" s="2">
+        <v>2.0600000000000001</v>
+      </c>
+      <c s="2">
+        <v>2.0899999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI76" s="2">
+        <v>1.3100000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.4399999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI77" s="2">
+        <v>1.03</v>
+      </c>
+      <c s="2">
+        <v>1.22</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI78" s="2">
+        <v>1.6100000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.77</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI79" s="2">
+        <v>1.52</v>
+      </c>
+      <c s="2">
+        <v>1.6000000000000001</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI80" s="2">
+        <v>1.1100000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.1299999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI81" s="2">
+        <v>0.84999999999999998</v>
+      </c>
+      <c s="2">
+        <v>1.0600000000000001</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI82" s="2">
+        <v>1.2</v>
+      </c>
+      <c s="2">
+        <v>1.3799999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI83" s="2">
+        <v>1.0900000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.24</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI84" s="2">
+        <v>1.27</v>
+      </c>
+      <c s="2">
+        <v>1.29</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI85" s="2">
+        <v>2.0600000000000001</v>
+      </c>
+      <c s="2">
+        <v>2.0800000000000001</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI86" s="2">
+        <v>1.21</v>
+      </c>
+      <c s="2">
+        <v>1.3100000000000001</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI87" s="2">
+        <v>0.77000000000000002</v>
+      </c>
+      <c s="2">
+        <v>0.81999999999999995</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI88" s="2">
+        <v>1.0600000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.28</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI89" s="2">
+        <v>1.02</v>
+      </c>
+      <c s="2">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI90" s="2">
+        <v>1</v>
+      </c>
+      <c s="2">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI91" s="2">
+        <v>1.47</v>
+      </c>
+      <c s="2">
+        <v>1.51</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI92" s="2">
+        <v>0.96999999999999997</v>
+      </c>
+      <c s="2">
+        <v>1.1299999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI93" s="2">
+        <v>1.7</v>
+      </c>
+      <c s="2">
+        <v>1.8400000000000001</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI94" s="2">
+        <v>1.78</v>
+      </c>
+      <c s="2">
+        <v>1.9399999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI95" s="2">
+        <v>0.93000000000000005</v>
+      </c>
+      <c s="2">
+        <v>1.3200000000000001</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI96" s="2">
+        <v>0.92000000000000004</v>
+      </c>
+      <c s="2">
+        <v>1.3600000000000001</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI97" s="2">
+        <v>1.5900000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.8799999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI98" s="2">
+        <v>0.68000000000000005</v>
+      </c>
+      <c s="2">
+        <v>0.72999999999999998</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI99" s="2">
+        <v>0.69999999999999996</v>
+      </c>
+      <c s="2">
+        <v>0.78000000000000003</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI100" s="2">
+        <v>1.0800000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.01</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI101" s="2">
+        <v>0.82999999999999996</v>
+      </c>
+      <c s="2">
+        <v>0.90000000000000002</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI102" s="2">
+        <v>1.1699999999999999</v>
+      </c>
+      <c s="2">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI103" s="2">
+        <v>0.97999999999999998</v>
+      </c>
+      <c s="2">
+        <v>0.95999999999999996</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI104" s="2">
+        <v>0.77000000000000002</v>
+      </c>
+      <c s="2">
+        <v>0.60999999999999999</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI105" s="2">
+        <v>0.91000000000000003</v>
+      </c>
+      <c s="2">
+        <v>1.27</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI106" s="2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c s="2">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI107" s="2">
+        <v>0.80000000000000004</v>
+      </c>
+      <c s="2">
+        <v>1.1200000000000001</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI108" s="2">
+        <v>0.84999999999999998</v>
+      </c>
+      <c s="2">
+        <v>0.71999999999999997</v>
+      </c>
+    </row>
+    <row>
+      <c r="AI109" s="2">
+        <v>0.81999999999999995</v>
+      </c>
+      <c s="2">
+        <v>0.87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#1395: Include Iain's updated test.xlsx.
</commit_message>
<xml_diff>
--- a/StatsDirectUI/Assets/Data/test.xlsx
+++ b/StatsDirectUI/Assets/Data/test.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fileVersion appName="SpreadsheetGear 7.4.12.102"/>
+  <fileVersion appName="SpreadsheetGear 8.0.65.102"/>
   <workbookPr defaultThemeVersion="153222"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="17340" windowHeight="11070" tabRatio="757"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1353" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1363" uniqueCount="544">
   <si>
     <t>2nd</t>
   </si>
@@ -1626,6 +1626,36 @@
   </si>
   <si>
     <t>Age (Years)</t>
+  </si>
+  <si>
+    <t>Venezuela</t>
+  </si>
+  <si>
+    <t>Colombia</t>
+  </si>
+  <si>
+    <t>Ecuador</t>
+  </si>
+  <si>
+    <t>Peru</t>
+  </si>
+  <si>
+    <t>Bolivia</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>GNP per capita</t>
+  </si>
+  <si>
+    <t>Infant Deaths</t>
+  </si>
+  <si>
+    <t>Live Births</t>
+  </si>
+  <si>
+    <t>Infant Mortality Rate (IMR)</t>
   </si>
 </sst>
 </file>
@@ -1668,38 +1698,10 @@
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF7F7F7F"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri Light"/>
-      <scheme val="major"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1707,9 +1709,13 @@
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF3F3F76"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1719,8 +1725,9 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1735,6 +1742,19 @@
       <name val="Arial"/>
     </font>
     <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri Light"/>
+      <scheme val="major"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF006100"/>
       <name val="Arial"/>
@@ -1743,6 +1763,16 @@
       <b/>
       <sz val="10"/>
       <color theme="0"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -1780,10 +1810,10 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5135,7 +5165,7 @@
       <c s="1">
         <v>2</v>
       </c>
-      <c s="9">
+      <c s="10">
         <v>35490</v>
       </c>
       <c s="2">
@@ -5185,7 +5215,7 @@
       <c s="1">
         <v>1</v>
       </c>
-      <c s="9">
+      <c s="10">
         <v>35552</v>
       </c>
       <c s="2">
@@ -5235,7 +5265,7 @@
       <c s="1">
         <v>1</v>
       </c>
-      <c s="9">
+      <c s="10">
         <v>35411</v>
       </c>
       <c s="2">
@@ -5285,7 +5315,7 @@
       <c s="1">
         <v>0</v>
       </c>
-      <c s="9">
+      <c s="10">
         <v>35370</v>
       </c>
       <c s="2">
@@ -5335,7 +5365,7 @@
       <c s="1">
         <v>2</v>
       </c>
-      <c s="9">
+      <c s="10">
         <v>35433</v>
       </c>
       <c s="2">
@@ -5383,7 +5413,7 @@
       <c s="1">
         <v>1</v>
       </c>
-      <c s="9">
+      <c s="10">
         <v>35555</v>
       </c>
       <c s="2">
@@ -5431,7 +5461,7 @@
       <c s="1">
         <v>0</v>
       </c>
-      <c s="9">
+      <c s="10">
         <v>35649</v>
       </c>
       <c s="2">
@@ -5479,7 +5509,7 @@
       <c s="1">
         <v>2</v>
       </c>
-      <c s="9">
+      <c s="10">
         <v>35346</v>
       </c>
       <c s="2">
@@ -10186,7 +10216,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AL805"/>
+  <dimension ref="A1:AQ805"/>
   <sheetFormatPr defaultColWidth="10.140625" defaultRowHeight="14.95"/>
   <cols>
     <col min="1" max="1" width="10" style="1" bestFit="1" customWidth="1"/>
@@ -10217,7 +10247,12 @@
     <col min="36" max="36" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="4.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="6" style="2" bestFit="1" customWidth="1"/>
-    <col min="39" max="16384" width="10.140625" style="2"/>
+    <col min="39" max="39" width="9.32421875" style="2" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="13.03125" style="2" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="22.21484375" style="2" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="8.87890625" style="2" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="11.62890625" style="2" bestFit="1" customWidth="1"/>
+    <col min="44" max="16384" width="10.140625" style="2"/>
   </cols>
   <sheetData>
     <row>
@@ -10335,6 +10370,21 @@
       <c s="2" t="s">
         <v>520</v>
       </c>
+      <c s="2" t="s">
+        <v>539</v>
+      </c>
+      <c s="2" t="s">
+        <v>540</v>
+      </c>
+      <c s="2" t="s">
+        <v>543</v>
+      </c>
+      <c s="2" t="s">
+        <v>542</v>
+      </c>
+      <c s="2" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -10451,6 +10501,21 @@
       <c s="2">
         <v>222.59999999999999</v>
       </c>
+      <c s="2" t="s">
+        <v>538</v>
+      </c>
+      <c s="2">
+        <v>2860</v>
+      </c>
+      <c s="2">
+        <v>59</v>
+      </c>
+      <c s="2">
+        <v>250</v>
+      </c>
+      <c s="2">
+        <v>14750</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -10567,6 +10632,21 @@
       <c s="2">
         <v>176.40000000000001</v>
       </c>
+      <c s="2" t="s">
+        <v>537</v>
+      </c>
+      <c s="2">
+        <v>4410</v>
+      </c>
+      <c s="2">
+        <v>43</v>
+      </c>
+      <c s="2">
+        <v>621</v>
+      </c>
+      <c s="2">
+        <v>26703</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -10683,6 +10763,21 @@
       <c s="2">
         <v>173.59999999999999</v>
       </c>
+      <c s="2" t="s">
+        <v>536</v>
+      </c>
+      <c s="2">
+        <v>4730</v>
+      </c>
+      <c s="2">
+        <v>39</v>
+      </c>
+      <c s="2">
+        <v>308</v>
+      </c>
+      <c s="2">
+        <v>12012</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -10799,6 +10894,21 @@
       <c s="2">
         <v>162.40000000000001</v>
       </c>
+      <c s="2" t="s">
+        <v>535</v>
+      </c>
+      <c s="2">
+        <v>6720</v>
+      </c>
+      <c s="2">
+        <v>24</v>
+      </c>
+      <c s="2">
+        <v>889</v>
+      </c>
+      <c s="2">
+        <v>21336</v>
+      </c>
     </row>
     <row>
       <c s="1">
@@ -10905,6 +11015,21 @@
       </c>
       <c s="2">
         <v>157.19999999999999</v>
+      </c>
+      <c s="2" t="s">
+        <v>534</v>
+      </c>
+      <c s="2">
+        <v>8130</v>
+      </c>
+      <c s="2">
+        <v>22</v>
+      </c>
+      <c s="2">
+        <v>568</v>
+      </c>
+      <c s="2">
+        <v>12496</v>
       </c>
     </row>
     <row>
@@ -47284,7 +47409,7 @@
       <c s="2">
         <v>1</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36179</v>
       </c>
       <c s="2">
@@ -47396,7 +47521,7 @@
       <c s="2">
         <v>3</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36193</v>
       </c>
       <c s="2">
@@ -47508,7 +47633,7 @@
       <c s="2">
         <v>5</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36207</v>
       </c>
       <c s="2">
@@ -47620,7 +47745,7 @@
       <c s="2">
         <v>7</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36221</v>
       </c>
       <c s="2">
@@ -47732,7 +47857,7 @@
       <c s="2">
         <v>9</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36235</v>
       </c>
       <c s="2">
@@ -47832,7 +47957,7 @@
       <c s="2">
         <v>11</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36249</v>
       </c>
       <c s="2">
@@ -47932,7 +48057,7 @@
       <c s="2">
         <v>13</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36263</v>
       </c>
       <c s="2">
@@ -48032,7 +48157,7 @@
       <c s="2">
         <v>15</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36277</v>
       </c>
       <c s="2">
@@ -48133,7 +48258,7 @@
       <c s="2">
         <v>17</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36291</v>
       </c>
     </row>
@@ -48215,7 +48340,7 @@
       <c s="2">
         <v>19</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36305</v>
       </c>
     </row>
@@ -48280,7 +48405,7 @@
       <c s="2">
         <v>21</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36319</v>
       </c>
     </row>
@@ -48341,7 +48466,7 @@
       <c s="2">
         <v>23</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36326</v>
       </c>
     </row>
@@ -48402,7 +48527,7 @@
       <c s="2">
         <v>25</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36354</v>
       </c>
     </row>
@@ -48463,7 +48588,7 @@
       <c s="2">
         <v>27</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36368</v>
       </c>
     </row>
@@ -48510,7 +48635,7 @@
       <c s="2">
         <v>29</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36382</v>
       </c>
     </row>
@@ -48557,7 +48682,7 @@
       <c s="2">
         <v>31</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36389</v>
       </c>
     </row>
@@ -48604,7 +48729,7 @@
       <c s="2">
         <v>33</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36417</v>
       </c>
     </row>
@@ -48639,7 +48764,7 @@
       <c s="2">
         <v>35</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36424</v>
       </c>
     </row>
@@ -48674,7 +48799,7 @@
       <c s="2">
         <v>37</v>
       </c>
-      <c s="10">
+      <c s="9">
         <v>36438</v>
       </c>
     </row>

</xml_diff>